<commit_message>
Add manufacturing pricing sheet to Excel and JSON baseline
Co-authored-by: phsayed2014-oss <phsayed2014-oss@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/exports/nostri-h1-2026-strategy-data.xlsx
+++ b/exports/nostri-h1-2026-strategy-data.xlsx
@@ -10,6 +10,7 @@
     <sheet name="كل الصيدليات H1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="المجمعات ص1 ص7 ص18" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="مستهدف 14 منتج" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="تسعير التصنيع" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -79,7 +80,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -87,6 +88,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -717,7 +719,6 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
@@ -740,7 +741,6 @@
       <c r="G10" s="3" t="n"/>
       <c r="H10" s="3" t="n"/>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
@@ -1010,7 +1010,6 @@
         <v>37.1</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
@@ -1495,64 +1494,653 @@
         <v>1000000</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>ترخيص صنف</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>6000</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>× 14</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>84000</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>تكلفة التصنيع</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>لاحقاً</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>هدف المجمعات 400K</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>ص1 ~180K</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>ص18 ~140K</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>ص7 ~80K</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>المنتج</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>تكلفة/حبة</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>MOQ</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>سعر البيع (80%)</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>ربح/حبة</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>تكلفة MOQ</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>إيراد MOQ</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>ربح MOQ</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>مستهدف شهري</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>وحدات/شهر</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Baby Shampoo</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>30000</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>150000</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>120000</v>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>65000</v>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Gel for Edema</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>50000</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>250000</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>200000</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>70000</v>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>1400</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Multivitamin</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>30000</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>150000</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>120000</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>85000</v>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>1700</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Mouth Wash HA</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>50000</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>250000</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>200000</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>70000</v>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>1400</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Mouth Wash H2O2</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>30000</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>150000</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>120000</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>65000</v>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Whitening Cream</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>45000</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>225000</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>180000</v>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>80000</v>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>1066.7</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Vitamin C</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>50000</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>250000</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>200000</v>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>60000</v>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Vitamin C + Zn</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>55000</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>275000</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>220000</v>
+      </c>
+      <c r="I9" s="2" t="n">
+        <v>70000</v>
+      </c>
+      <c r="J9" s="2" t="n">
+        <v>1272.7</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Strepsils Menthol</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>60000</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>300000</v>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I10" s="2" t="n">
+        <v>75000</v>
+      </c>
+      <c r="J10" s="2" t="n">
+        <v>1250</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Strepsils Honey &amp; Lemon</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>60000</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>300000</v>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I11" s="2" t="n">
+        <v>70000</v>
+      </c>
+      <c r="J11" s="2" t="n">
+        <v>1166.7</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Zn Syrup</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>45000</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>225000</v>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>180000</v>
+      </c>
+      <c r="I12" s="2" t="n">
+        <v>65000</v>
+      </c>
+      <c r="J12" s="2" t="n">
+        <v>866.7</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Vit D Drops</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>45000</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>225000</v>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>180000</v>
+      </c>
+      <c r="I13" s="2" t="n">
+        <v>60000</v>
+      </c>
+      <c r="J13" s="2" t="n">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Vision Tablet</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>45000</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>225000</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>180000</v>
+      </c>
+      <c r="I14" s="2" t="n">
+        <v>75000</v>
+      </c>
+      <c r="J14" s="2" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Natal / Pregnatabs</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>45000</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>225000</v>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>180000</v>
+      </c>
+      <c r="I15" s="2" t="n">
+        <v>90000</v>
+      </c>
+      <c r="J15" s="2" t="n">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>الإجمالي</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>640000</v>
+      </c>
+      <c r="G16" s="5" t="n">
+        <v>3200000</v>
+      </c>
+      <c r="H16" s="5" t="n">
+        <v>2560000</v>
+      </c>
+    </row>
     <row r="17"/>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ترخيص صنف</t>
+          <t>ترخيص 14×6000</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>6000</v>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>× 14</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
         <v>84000</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>تكلفة التصنيع</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>لاحقاً</t>
-        </is>
-      </c>
-    </row>
-    <row r="20"/>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>هدف المجمعات 400K</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>ص1 ~180K</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>ص18 ~140K</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>ص7 ~80K</t>
-        </is>
+          <t>أقصى نقدي MOQ+ترخيص</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>724000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>